<commit_message>
Finalize Level 3 lessons 3.1-3.6 (reviewed and verified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/03-data-analysis/03-data-cleaning/3.3-data-cleaning.xlsx
+++ b/03-data-analysis/03-data-cleaning/3.3-data-cleaning.xlsx
@@ -1208,11 +1208,11 @@
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>TRIM removes leading and trailing spaces and shrinks inner runs to one space, so any name it shortens had extra spaces. Comparing lengths tests all 650 rows at once: the comparison gives TRUE/FALSE for each row, the double minus turns those into 1/0, and SUMPRODUCT adds them. You can't see a trailing space by looking at a cell, so a count like this is how you find out a problem exists before you fix it. (In Microsoft 365, =SUM(--(LEN(…)&lt;&gt;LEN(TRIM(…)))) works too.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="111" customHeight="1">
+          <t>TRIM removes leading and trailing spaces and shrinks inner runs to one space, so any name it shortens had extra spaces. Comparing lengths tests all 650 rows at once: the comparison gives TRUE/FALSE for each row, the double minus turns those into 1/0, and SUMPRODUCT adds them. You can't see a trailing space by looking at a cell, so a count like this is how you find out a problem exists before you fix it. In Microsoft 365, =SUM(--(LEN(…)&lt;&gt;LEN(TRIM(…)))) works too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="126" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>2</t>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="F6" s="19" t="inlineStr">
         <is>
-          <t>Every spelling starts with the right letter once the stray space is gone, so the fix is TRIM → LEFT(…,1) → UPPER. The order matters: LEFT(" F",1) is a space. The check uses EXACT because COUNTIF ignores case and would count a lowercase f as F. This shortcut works only because each value is identified by its first letter. Medicare and Medicaid share a first letter, so Insurance needs a mapping table instead (task 8).</t>
+          <t>Every spelling starts with the right letter once the stray space is gone, so the fix is TRIM, then LEFT(…,1), then UPPER. The order matters: LEFT(" F",1) is a space. The check uses EXACT because COUNTIF ignores case and would count a lowercase f as F. This shortcut works only because each value is identified by its first letter. Medicare and Medicaid share a first letter, so Insurance needs a mapping table instead (task 8).</t>
         </is>
       </c>
     </row>
@@ -1257,11 +1257,11 @@
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>1. Right-click the **Raw** tab → **Move or Copy…** → tick **Create a copy** → **OK**. Work on **Raw (2)**.
-2. Click any cell in the data, then **Data → Remove Duplicates**.
-3. Keep **My data has headers** ticked. Untick **RecordID** and leave the other nine columns ticked. Click **OK**.
-4. Excel reports *40 duplicate values found and removed; 610 unique values remain.*
-Formula check without deleting anything (Microsoft 365 / Excel 2021+): `=ROWS(Raw!B2:J651)-ROWS(UNIQUE(Raw!B2:J651))`</t>
+          <t>1. Right-click the Raw tab → Move or Copy… → tick Create a copy → OK. Work on Raw (2).
+2. Click any cell in the data, then Data → Remove Duplicates.
+3. Keep My data has headers ticked. Untick RecordID and leave the other nine columns ticked. Click OK.
+4. Excel reports 40 duplicate values found and removed; 610 unique values remain.
+Formula check without deleting anything (Microsoft 365 / Excel 2021+): =ROWS(Raw!B2:J651)-ROWS(UNIQUE(Raw!B2:J651))</t>
         </is>
       </c>
       <c r="E7" cm="1" s="41">
@@ -1290,12 +1290,12 @@
       </c>
       <c r="D8" s="40" t="inlineStr">
         <is>
-          <t>1. Select **A2:B50** on CensusExport (not the whole columns, and not the header row).
-2. **Home → Find &amp; Select → Go To Special…** (or press **F5**, Mac: **⌃ + G**, then **Special…**). Choose **Blanks** → **OK**. Only the empty cells stay selected.
-3. Without clicking anywhere, type **=** and press **↑**. The active cell is the first blank, A3, so the formula reads `=A2`.
-4. Press **Ctrl + Enter** (Mac: **⌘ + Return**) to put that formula in every selected blank. Each copy points to the cell above itself.
-5. Turn the formulas into values: select A2:B50, copy, then **Paste Special → Values**.
-Check with `=SUMIFS(CensusExport!E2:E50,CensusExport!A2:A50,"Cedar Ridge Medical Center",CensusExport!B2:B50,"Intensive Care Unit")`</t>
+          <t>1. Select A2:B50 on CensusExport (not the whole columns, and not the header row).
+2. Home → Find &amp; Select → Go To Special… (or press F5, Mac: ⌃ + G, then Special…). Choose Blanks → OK. Only the empty cells stay selected.
+3. Without clicking anywhere, type = and press ↑. The active cell is the first blank, A3, so the formula reads =A2.
+4. Press Ctrl + Enter (Mac: ⌘ + Return) to put that formula in every selected blank. Each copy points to the cell above itself.
+5. Turn the formulas into values: select A2:B50, copy, then Paste Special → Values.
+Check with =SUMIFS(CensusExport!E2:E50,CensusExport!A2:A50,"Cedar Ridge Medical Center",CensusExport!B2:B50,"Intensive Care Unit")</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
@@ -1325,11 +1325,11 @@
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
-          <t>1. In **O2** type **45501** (from *Bluestone OH 45501*), and in **O3** type **45720** (from *CEDAR RIDGE, OH 45720*).
-2. In the first ZIP+4 row, **O11** (*Bluestone, OH 45501-8106*), type **45501**.
-3. Select **O4**, the first empty cell, and press **Ctrl + E** (or **Data → Flash Fill**).
-4. Check the result: `=SUMPRODUCT(--(LEN(Clean!O2:O651)&lt;&gt;5))` should return 0. If some rows are wrong, press Ctrl + Z, type the correct ZIP on one of the wrong rows as an extra example, and run Flash Fill again.
-Formula alternative (Microsoft 365): `=LEFT(TEXTAFTER(G2," ",-1),5)`</t>
+          <t>1. In O2 type 45501 (from Bluestone OH 45501), and in O3 type 45720 (from CEDAR RIDGE, OH 45720).
+2. In the first ZIP+4 row, O11 (Bluestone, OH 45501-8106), type 45501.
+3. Select O4, the first empty cell, and press Ctrl + E (or Data → Flash Fill).
+4. Check the result: =SUMPRODUCT(--(LEN(Clean!O2:O651)&lt;&gt;5)) should return 0. If some rows are wrong, press Ctrl + Z, type the correct ZIP on one of the wrong rows as an extra example, and run Flash Fill again.
+Formula alternative (Microsoft 365): =LEFT(TEXTAFTER(G2," ",-1),5)</t>
         </is>
       </c>
       <c r="E9" cm="1" s="41">
@@ -1338,11 +1338,11 @@
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>Flash Fill looks for a rule that explains every example you typed. Two plain ZIPs fit several rules (the first number, the last number, the last five characters), and on 45501-8106 those give different answers. The ZIP+4 example leaves only "the first number". If the +4 survives, the distinct count jumps to 108. Flash Fill writes typed-in values, not formulas, so it won't update when next month's export arrives. In Lesson 2.2 you did the same job with TEXTAFTER. The formula is the repeatable choice, and Flash Fill is the fast one for a one-off.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="141" customHeight="1">
+          <t>Flash Fill looks for a rule that explains every example you typed. Two plain ZIPs fit several rules (the first number, the last number, the last five characters), and on 45501-8106 those give different answers. The ZIP+4 example leaves only "the first number". If the +4 survives, the distinct count jumps to 108. Flash Fill writes typed-in values, not formulas, so it won't update when next month's export arrives. The Lesson 2.2 bonus did the same job with TEXTAFTER. The formula is the repeatable choice, and Flash Fill is the fast one for a one-off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="156" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>6</t>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>Each SUBSTITUTE deletes one kind of character: parentheses, dashes, dots, and spaces. That leaves 5554767432 for most rows, but +15555973811 for the 40 numbers with a country code, so RIGHT(…,10) keeps the last ten digits, which is always the U.S. number. A blank phone stays empty, and the 30 blanks are why the count is 620, not 650. Keep phones as text: they are identifiers, not quantities. In Microsoft 365, =RIGHT(REGEXREPLACE(E2,"[^0-9]",""),10) removes every non-digit in one step.</t>
+          <t>Each SUBSTITUTE deletes one kind of character: parentheses, dashes, dots, and spaces. That leaves 5554767432 for most rows, but +15555973811 for the 40 numbers with a country code, so RIGHT(…,10) keeps the last ten digits, which is always the U.S. number. A blank phone needs no special handling, because SUBSTITUTE and RIGHT on an empty cell return an empty result. The 30 blanks are why the count is 620, not 650. Keep phones as text, because they are identifiers, not quantities. In Microsoft 365, =RIGHT(REGEXREPLACE(E2,"[^0-9]",""),10) removes every non-digit in one step.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>A mapping table turns a messy category into a standard code with one lookup, and it documents your decisions where everyone can see them, such as Uninsured → PY07 Self-Pay. XLOOKUP ignores case, so the map needs only one row per spelling, not one per capitalization. It does not ignore spaces, so TRIM comes first. Without TRIM, the 12 rows typed "Silverline Medicare Advantage " with a trailing space come back UNMAPPED. The "UNMAPPED" result makes new spellings easy to find next month: filter for it, add the spelling as a new row of the map, and every formula picks it up. The Table references (tblPayerMap[Variant]) grow with the map. A fixed range such as PayerMap!$A$2:$A$20 works today but would miss a row added below it. Without XLOOKUP: =IFNA(VLOOKUP(TRIM(H2),tblPayerMap,2,FALSE),"UNMAPPED").</t>
+          <t>A mapping table turns a messy category into a standard code with one lookup, and it documents your decisions where everyone can see them, such as the rule that Uninsured means PY07 (Self-Pay). XLOOKUP ignores case, so the map needs only one row per spelling, not one per capitalization. It does not ignore spaces, so TRIM comes first. Without TRIM, the 12 rows typed "Silverline Medicare Advantage " with a trailing space come back UNMAPPED. The "UNMAPPED" result makes new spellings easy to find next month: filter for it, add the spelling as a new row of the map, and every formula picks it up. The Table references (tblPayerMap[Variant]) grow with the map. A fixed range such as PayerMap!$A$2:$A$20 works today but would miss a row added below it. Without XLOOKUP, use =IFNA(VLOOKUP(TRIM(H2),tblPayerMap,2,FALSE),"UNMAPPED").</t>
         </is>
       </c>
     </row>
@@ -1445,11 +1445,11 @@
       </c>
       <c r="D13" s="40" t="inlineStr">
         <is>
-          <t>1. On **LabFeed**, select **A1:A117** (header included).
-2. **Data → Text to Columns**. Choose **Delimited** → **Next**.
-3. Untick **Tab**, tick **Other**, and type a vertical bar **|** in the box. The preview splits into five columns. Click **Next**.
-4. Click the **MRN** column in the preview and choose **Text** as its column data format. Optionally click the last column and choose **Date: MDY**. Click **Finish**.
-Check with `=AVERAGEIF(LabFeed!B2:B117,"K",LabFeed!C2:C117)`</t>
+          <t>1. On LabFeed, select A1:A117 (header included).
+2. Data → Text to Columns. Choose Delimited → Next.
+3. Untick Tab, tick Other, and type a vertical bar | in the box. The preview splits into five columns. Click Next.
+4. Click the MRN column in the preview and choose Text as its column data format. Optionally click the last column and choose Date: MDY. Click Finish.
+Check with =AVERAGEIF(LabFeed!B2:B117,"K",LabFeed!C2:C117)</t>
         </is>
       </c>
       <c r="E13" cm="1" s="43">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Fill the yellow NameClean column (K) with every name as First Last in Proper Case, with single spaces: "Haddad, Jonathan" → Jonathan Haddad, "  Alexander ,  Gary " → Gary Alexander, and "Amber White" stays Amber White. 92 rows are already First Last (no comma). The gray cell warns if any name still has extra spaces or is ALL CAPS or all lowercase. Otherwise it counts distinct names.</t>
+          <t>Fill the yellow NameClean column (K) with every name as First Last in Proper Case, with single spaces. For example, "Haddad, Jonathan" becomes Jonathan Haddad, "  Alexander ,  Gary " becomes Gary Alexander, and "Amber White" stays Amber White. 92 rows are already First Last (no comma). The gray cell warns if any name still has extra spaces or is ALL CAPS or all lowercase. Otherwise it counts distinct names.</t>
         </is>
       </c>
       <c r="C14" s="39" t="n">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>FIND(",",B2) returns a position when there is a comma and #VALUE! when there isn't, so ISNUMBER(FIND(…)) tells the two layouts apart. For Last, First rows, MID takes everything after the comma (the first name) and LEFT takes everything before it (the last name). TRIM each piece before joining, because the spaces sit around the comma. PROPER on the outside fixes the case of both layouts at once. Two checks on the result. First, the flip matters: =PROPER(TRIM(B2)) alone gives 578 distinct names, and deleting the comma without flipping still gives 569, because the same patient then appears as both "Amber White" (row 18) and "White Amber" (row 410). Second, the count is 557, not 560, because 3 names belong to two different patients (Justin Lewis, Lisa Morris, Mei Myers). That's why you dedupe on MRN, never on name. PROPER also turns McDonald into Mcdonald, so fix known exceptions by hand and note them in the cleaning log.</t>
+          <t>FIND(",",B2) returns a position when there is a comma and #VALUE! when there isn't, so ISNUMBER(FIND(…)) tells the two layouts apart. For Last, First rows, MID takes everything after the comma (the first name) and LEFT takes everything before it (the last name). TRIM each piece before joining, because the spaces sit around the comma. PROPER on the outside fixes the case of both layouts at once. Two checks on the result. First, the flip matters: =PROPER(TRIM(B2)) alone gives 578 distinct names, and deleting the comma without flipping still gives 569, because the same patient then appears as both "Amber White" (row 18) and "White Amber" (row 410). Second, the count is 557, not 560, because 3 names belong to two different patients (Justin Lewis, Lisa Morris, Mei Myers). That's why you deduplicate on MRN, never on name. PROPER also turns McDonald into Mcdonald, so fix known exceptions by hand and note them in the cleaning log.</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="111" customHeight="1">
+    <row r="16" ht="126" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>12</t>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>A cleaning log records what you changed and how much, so the next person (or you, next month) can repeat it and audit it. "Rows changed" is the most useful number in it: here 424 of 650 rows changed and 226 were already F or M. EXACT matters again: with =, "f" equals "F" and those rows would look unchanged. A count that is suspiciously high or low is often the first sign that a cleaning formula is wrong.</t>
+          <t>A cleaning log records what you changed and how much, so the next person (or you, next month) can repeat it and audit it. "Rows changed" is the most useful number in it: here 424 of 650 rows changed and 226 were already F or M. EXACT matters again, because with = the values "f" and "F" count as equal and those rows would look unchanged. A count that is suspiciously high or low is often the first sign that a cleaning formula is wrong.</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="126" customHeight="1">
+    <row r="5" ht="141" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>B1</t>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>Both layouts put the time at character 12, so TIMEVALUE(MID(J2,12,8)) reads "18:33:00" and "05:42 PM" alike, and AM/PM is handled for you. The date part differs, so the IF builds it with DATE from the right pieces. A date-time is just date + time (a whole number plus a fraction of a day). If PM were ignored, the evening count would drop to 76. With U.S. regional settings, =--J2 (or =VALUE(J2)) converts both layouts in one step.</t>
+          <t>Both layouts put the time at character 12, so TIMEVALUE(MID(J2,12,8)) reads "18:33:00" and "05:42 PM" alike, and AM/PM is handled for you. The date part differs, so the IF builds it with DATE from the right pieces. In the ISO layout the day is MID(J2,9,2), not RIGHT(J2,2), because the time follows it. A date-time is just date + time (a whole number plus a fraction of a day). If PM were ignored, the evening count would drop to 76. With U.S. regional settings, =--J2 (or =VALUE(J2)) converts both layouts in one step.</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="F6" s="19" t="inlineStr">
         <is>
-          <t>The first test, RegisteredClean = MAXIFS(all RegisteredClean, all MRNClean, this MRN), is TRUE on the patient's latest row. Exact copies share that time, so the second test counts how many rows so far (the range $Q$2:Q2 grows as the formula goes down) have this MRN and this time. It equals 1 only on the first of them. The total must equal the 560 distinct MRNs from practice task 7, which is a good cross-check. Avoid comparing date-times with "&gt;"&amp;R2 inside COUNTIFS: that turns the time into text with 15 digits and can miss by a rounding error.</t>
+          <t>The first test, RegisteredClean = MAXIFS(all RegisteredClean, all MRNClean, this MRN), is TRUE on the patient's latest row. Exact copies share that time, so the second test counts how many rows so far (the range $Q$2:Q2 grows as the formula goes down) have this MRN and this time. It equals 1 only on the first of them. The total must equal the 560 distinct MRNs from practice task 7, which is a good cross-check. Avoid comparing date-times with "&gt;"&amp;R2 inside COUNTIFS, because that turns the time into text with 15 digits and can miss by a rounding error.</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="141" customHeight="1">
+    <row r="9" ht="171" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>B5</t>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Survivorship check: "keep the latest row" can throw away good data. How many kept rows have an empty PhoneClean even though another registration for the same patient has a phone number?</t>
+          <t>The rule "keep the latest row" decides which registration survives into the master list, and it can throw away good data. How many kept rows have an empty PhoneClean even though another registration for the same patient has a phone number?</t>
         </is>
       </c>
       <c r="C9" s="39" t="n">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>When its criteria argument is a range instead of a single value, COUNTIFS returns one count per row: how many rows share this row's MRN and have a phone. "?*" means at least one character, which works because PhoneClean is text. Multiply by Keep and by an empty PhoneClean to find the 2 patients who would arrive in the new EHR with no phone, although an older registration has one. Real MPI loads use survivorship rules for this: take each field from the most recent row that has it filled in, not every field from the most recent row.</t>
+          <t>When its criteria argument is a range instead of a single value, COUNTIFS returns one count per row: how many rows share this row's MRN and have a phone. The criteria "?*" means at least one character, which works because PhoneClean is text. Multiply by Keep and by an empty PhoneClean to find the 2 patients who would arrive in the new EHR with no phone, although an older registration has one. Real master patient index (MPI) loads prevent this with survivorship rules, which decide field by field which value survives. A common rule takes each field from the most recent row that has it filled in, instead of taking every field from the most recent row.</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Go To Special selects only the blanks; Ctrl + Enter fills them all with one relative formula</t>
+          <t>Go To Special selects only the blanks, and Ctrl + Enter fills them all with one relative formula</t>
         </is>
       </c>
       <c r="D9" cm="1" s="23">
@@ -2069,7 +2069,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="81" customHeight="1">
+    <row r="15" ht="96" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
           <t>10</t>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Fill the yellow NameClean column (K) with every name as First Last in Proper Case, with single spaces: "Haddad, Jonathan" → Jonathan Haddad, "  Alexander ,  Gary " → Gary Alexander, and "Amber White" stays Amber White. 92 rows are already First Last (no comma). The gray cell warns if any name still has extra spaces or is ALL CAPS or all lowercase. Otherwise it counts distinct names.</t>
+          <t>Fill the yellow NameClean column (K) with every name as First Last in Proper Case, with single spaces. For example, "Haddad, Jonathan" becomes Jonathan Haddad, "  Alexander ,  Gary " becomes Gary Alexander, and "Amber White" stays Amber White. 92 rows are already First Last (no comma). The gray cell warns if any name still has extra spaces or is ALL CAPS or all lowercase. Otherwise it counts distinct names.</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
-          <t>EXACT compares case-sensitively; NOT flips it; SUMPRODUCT(--…) counts</t>
+          <t>EXACT compares case-sensitively, NOT flips TRUE and FALSE, and SUMPRODUCT(--…) counts the TRUEs</t>
         </is>
       </c>
       <c r="D17" cm="1" s="23">
@@ -76046,7 +76046,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Leading zeros lost on some rows; MRN- prefix on others</t>
+          <t>Leading zeros lost on some rows, and an MRN- prefix on others</t>
         </is>
       </c>
       <c r="D6" s="33" t="n"/>
@@ -76167,7 +76167,7 @@
     <row r="2" ht="64" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Bluestone is moving to a new EHR, and the vendor needs a master patient load file with exactly one row per patient. The rule from Patient Access is: keep each patient's most recent registration (latest RegisteredOn). Work on the Clean sheet's last two yellow columns (RegisteredClean and Keep), using your MRNClean and PhoneClean columns from the practice tasks, then answer on the Bonus sheet. RegisteredOn has two layouts: 2015-11-06 18:33:00 (24-hour clock) and 05/30/2022 05:42 PM (12-hour clock).</t>
+          <t>Bluestone is moving to a new EHR, and the vendor needs a master patient load file with exactly one row per patient. The rule from Patient Access is: keep each patient's most recent registration (latest RegisteredOn). Fill the Clean sheet's last two yellow columns (RegisteredClean and Keep), using your MRNClean and PhoneClean columns from the practice tasks. RegisteredOn has two layouts: 2015-11-06 18:33:00 (24-hour clock) and 05/30/2022 05:42 PM (12-hour clock). If you want helper columns, put them on the Clean sheet in column V or further right, outside the Table.</t>
         </is>
       </c>
     </row>
@@ -76224,7 +76224,7 @@
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>In both layouts the time starts at character 12, and TIMEVALUE understands both 18:33:00 and 05:42 PM. Build the date part with DATE</t>
+          <t>In both layouts the time starts at character 12, and TIMEVALUE understands both 18:33:00 and 05:42 PM. Build the date part with DATE, then add the time to it</t>
         </is>
       </c>
       <c r="D6" cm="1" s="23">
@@ -76249,7 +76249,7 @@
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>MAXIFS finds the patient's latest time. A COUNTIFS over an expanding range ($Q$2:Q2) breaks ties</t>
+          <t>MAXIFS (Lesson 2.5) finds the patient's latest time. A COUNTIFS over an expanding range ($Q$2:Q2) breaks ties</t>
         </is>
       </c>
       <c r="D7" cm="1" s="23">
@@ -76261,7 +76261,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="66" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>B3</t>
@@ -76274,7 +76274,7 @@
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>MAXIFS (or XLOOKUP) with two conditions: this MRN, and Keep = TRUE</t>
+          <t>MAXIFS with two conditions: MRNClean is this MRN, and Keep is TRUE. Or filter Clean on those two columns and read RegisteredClean</t>
         </is>
       </c>
       <c r="D8" s="35" t="n"/>
@@ -76296,7 +76296,7 @@
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>A row is a patient's first occurrence when MATCH(its MRN, the MRN column, 0) returns its own position. Or add a helper column with COUNTIF($Q$2:Q2,Q2)=1</t>
+          <t>A row is a patient's first occurrence when MATCH(its MRN, the MRN column, 0) returns its own position. Or add a helper column with =COUNTIF($Q$2:Q2,Q2)=1</t>
         </is>
       </c>
       <c r="D9" s="21" t="n"/>
@@ -76305,7 +76305,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="51" customHeight="1">
+    <row r="10" ht="66" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>B5</t>
@@ -76313,7 +76313,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Survivorship check: "keep the latest row" can throw away good data. How many kept rows have an empty PhoneClean even though another registration for the same patient has a phone number?</t>
+          <t>The rule "keep the latest row" decides which registration survives into the master list, and it can throw away good data. How many kept rows have an empty PhoneClean even though another registration for the same patient has a phone number?</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">

</xml_diff>